<commit_message>
Revised various adaptors, Updated Reference Board
Reference board has an additional degree of freedom for input beam, changed geometry for everything else
</commit_message>
<xml_diff>
--- a/Production/Laser_Board/Laser_Board2.xlsx
+++ b/Production/Laser_Board/Laser_Board2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Github/PyOpticL_Rubidium_System/Production/LaserBoard2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kim/Desktop/Lab/Sinclair/pyopticl-setups/Production/Laser_Board/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BCD92B5-3AA7-9948-872C-09F5741A28FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48C9A58-3CBC-0A4D-8BA2-66FC281EF21C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
+    <workbookView xWindow="14700" yWindow="660" windowWidth="14700" windowHeight="16680" xr2:uid="{42F6A15E-87CE-9147-9545-45C46C70D310}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>Adaptors</t>
   </si>
@@ -76,15 +76,6 @@
     <t>Elements</t>
   </si>
   <si>
-    <t>IOT-5-850-MP</t>
-  </si>
-  <si>
-    <t>cube</t>
-  </si>
-  <si>
-    <t>Laser Board2</t>
-  </si>
-  <si>
     <t>KA05T</t>
   </si>
   <si>
@@ -94,14 +85,32 @@
     <t>IPS_adapter.step</t>
   </si>
   <si>
-    <t>Laser_Baseplate2.step</t>
+    <t>IOT-5-780-MP</t>
+  </si>
+  <si>
+    <t>PBS</t>
+  </si>
+  <si>
+    <t>Optics</t>
+  </si>
+  <si>
+    <t>QWP</t>
+  </si>
+  <si>
+    <t>HWP</t>
+  </si>
+  <si>
+    <t>Laser Board</t>
+  </si>
+  <si>
+    <t>Laser_Baseplate.step</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -115,6 +124,13 @@
       <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -139,9 +155,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -477,70 +503,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{504A0317-4413-EE44-9F8B-28AC1E65744B}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8">
+      <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9">
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="3">
         <v>1</v>
       </c>
     </row>
@@ -548,7 +575,7 @@
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>1</v>
       </c>
     </row>
@@ -556,92 +583,116 @@
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="B16" s="4">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="B17" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18">
+        <v>9</v>
+      </c>
+      <c r="B18" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="B19" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B20">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>14</v>
-      </c>
-      <c r="B22">
+      <c r="B26" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="4">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A18" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
-    <hyperlink ref="A19" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
+    <hyperlink ref="A16" r:id="rId1" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05L05" xr:uid="{26D03288-5EB5-E849-A9E7-78F166728512}"/>
+    <hyperlink ref="A17" r:id="rId2" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=SM05FCA2" xr:uid="{7396B97A-1E53-F246-B983-DFB7235DDE2B}"/>
     <hyperlink ref="A15" r:id="rId3" xr:uid="{1BBCBD75-E5E4-9C42-9870-10D5AFE8751D}"/>
     <hyperlink ref="A13" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=RSP05" xr:uid="{8DD89EFB-A6D7-DC45-81DC-A3DF706D2C18}"/>
-    <hyperlink ref="A20" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
-    <hyperlink ref="A21" r:id="rId6" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
-    <hyperlink ref="A16" r:id="rId7" xr:uid="{103D64FF-9059-1B42-816A-F92B0274781E}"/>
-    <hyperlink ref="A17" r:id="rId8" xr:uid="{6F72CF33-8356-4942-9395-81A746EF906E}"/>
+    <hyperlink ref="A26" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=BB05-E03" xr:uid="{A85C602C-A7C0-4B48-94F9-6B38884C0FD3}"/>
+    <hyperlink ref="A18" r:id="rId6" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=S05TM09" xr:uid="{EF391373-8D5D-B54F-B9A3-5D87DFC3B5D2}"/>
+    <hyperlink ref="A20" r:id="rId7" xr:uid="{103D64FF-9059-1B42-816A-F92B0274781E}"/>
+    <hyperlink ref="A19" r:id="rId8" xr:uid="{6F72CF33-8356-4942-9395-81A746EF906E}"/>
     <hyperlink ref="A14" r:id="rId9" xr:uid="{CD36AEA7-5080-754C-810A-7239C2468B80}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>